<commit_message>
docs: visual update clockify
</commit_message>
<xml_diff>
--- a/docs/Sprint 3/Clockify.xlsx
+++ b/docs/Sprint 3/Clockify.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sergi\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sergi\Desktop\ISPP-G8\ISPP-G8\docs\Sprint 3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C764BD9C-E02C-47BF-8B5F-77A76556590F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C5383A3-D397-4CFA-B82E-BED2916C5F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -288,7 +288,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -318,28 +318,52 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1" tint="0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -362,16 +386,63 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -384,10 +455,41 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -964,7 +1066,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="es-ES"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1018,7 +1120,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E5232C7B-A338-43EC-A13D-3B83B2FF3288}" type="CELLRANGE">
+                    <a:fld id="{39C84226-08D9-4957-819C-701A1E703EC0}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1036,7 +1138,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1051,8 +1152,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6AC52A7F-0E57-4A5B-A89C-A1898490981C}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{706351A4-728F-4320-8E6C-747EADEDEC08}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1084,8 +1185,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{469653E5-400E-4E0F-BF66-FBCC7A4A69B3}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{037EE795-49B1-4C37-862C-E9061CCB617B}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1117,8 +1218,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BD7A2A4A-6861-4F21-86A8-2E872C004A96}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{83759FE0-8D5C-4705-8A38-B59BF6DD68C5}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1150,8 +1251,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{42AD7C93-0466-4125-AD95-C22A3E70AC4C}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{D25EB1D6-D183-4927-B3E2-BFF0771A3FD3}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1183,8 +1284,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{619F6ED2-D50E-4B87-B03A-DC772F413CE5}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{D84FFE4F-479C-4D8A-A0F4-FB8D422E762C}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1216,8 +1317,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E9927F25-15FC-4F2A-A02F-5FCBF57C0950}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{BA754F38-D27A-4613-9B4E-C4016D4663D6}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1249,8 +1350,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F377ABE6-BFDB-4A40-B807-D74F64B7895B}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{10F2D0DF-CC04-4CDA-B7EF-80DDD19D3F2D}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1282,8 +1383,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8CBFC46B-7E94-44F2-9498-0049B5D52260}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{34FDDB7F-0F86-4FA5-80F3-550460F78023}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1315,8 +1416,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{05D859E9-9F7B-469E-8636-6C1391240347}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{133A516B-1C70-40CC-9C2E-2D041409A4A4}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1348,8 +1449,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{0D2CB055-6D2E-4288-ACB2-185BC04E2C07}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{C6569794-FCB8-486A-ACC1-6957B9BA360B}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1381,8 +1482,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FCDACCC1-9F85-422E-86A5-4CB1681D89F0}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{221F2421-6EA0-45BC-9757-60AFB7C82F61}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1414,8 +1515,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D7742880-0477-4C9F-AFBE-E7D13CBCF6DE}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{90D62DCE-948D-45F5-81A6-8ABCF15B4AC4}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1447,8 +1548,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{826FA39A-EAC9-40DA-AC38-613C4387E050}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{513F73E1-0717-4084-93C5-24CF85FFF94B}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1480,8 +1581,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F2C40098-26CD-40D8-BB2B-7B301FF5A9B6}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{9519F901-EDD3-4BAA-A557-D50A724E65C7}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1513,8 +1614,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{19A3C4E6-84D1-43A7-9AB1-50122F675D88}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{82E76E88-8738-419D-AC70-17B92DA20E88}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1546,8 +1647,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{3CE9341A-3D82-4A76-A85A-5BBD1FFBB227}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{45EF95D3-C754-4816-87D7-5B7ECDA447BD}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1579,8 +1680,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6278A0D3-1922-4972-BAC2-518A5E15106E}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{9C3E240C-C14D-4CC1-A93D-64A31FC0E802}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1612,8 +1713,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{566F64A6-9DE5-40C4-BC9D-8CE0B147456E}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{E2AE90D5-2C82-4C7D-9BE7-E41F6229702F}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -1645,8 +1746,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C15C7E12-CC5C-467D-B9BF-729B8F44FF4C}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{0C79F16E-DB81-438D-B8A5-94C501AA61CD}" type="CELLRANGE">
+                      <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
@@ -3307,16 +3408,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>23812</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>342900</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>100012</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>314325</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>80962</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3344,15 +3445,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>19049</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>14287</xdr:rowOff>
+      <xdr:colOff>609599</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>600074</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>581024</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3643,16 +3744,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.42578125" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
     <col min="4" max="4" width="18.7109375" customWidth="1"/>
-    <col min="5" max="5" width="26.42578125" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" customWidth="1"/>
     <col min="6" max="6" width="19.42578125" customWidth="1"/>
     <col min="7" max="7" width="17.140625" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" customWidth="1"/>
     <col min="9" max="10" width="9.140625" customWidth="1"/>
     <col min="12" max="12" width="9.140625" customWidth="1"/>
     <col min="18" max="18" width="21" customWidth="1"/>
@@ -3661,713 +3763,778 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="24" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="16" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="8">
         <v>0.29987268518518517</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="7">
         <v>0</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="7">
         <f>_xlfn.NORM.DIST(D2, C23, C24, FALSE)</f>
         <v>2.2218545233217101E-2</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="9">
         <f>C2*24</f>
         <v>7.1969444444444441</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="5">
         <v>8.9494907407407407</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="7" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="8">
         <v>0.98466435185185186</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="7">
         <v>1</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="7">
         <f>_xlfn.NORM.DIST(D3, C23, C2, FALSE)</f>
         <v>2.6983539181641642E-167</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="9">
         <f t="shared" ref="F3:F21" si="0">C3*24</f>
         <v>23.631944444444443</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="5">
         <v>6.9386574074074066</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="7" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="8">
         <v>0.35123842592592591</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="7">
         <v>2</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="7">
         <f>_xlfn.NORM.DIST(D4, C23, C24, FALSE)</f>
         <v>3.2693965909748872E-2</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="9">
         <f t="shared" si="0"/>
         <v>8.429722222222221</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="5">
         <v>9.1549537037037041</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="7" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="8">
         <v>0.6287962962962963</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="7">
         <v>3</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="7">
         <f>_xlfn.NORM.DIST(D5, C23, C24, FALSE)</f>
         <v>3.8300164745237071E-2</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="9">
         <f t="shared" si="0"/>
         <v>15.091111111111111</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="5">
         <v>6.5151851851851852</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="7" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="8">
         <v>0.25579861111111113</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="7">
         <v>4</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="7">
         <f>_xlfn.NORM.DIST(D6, C23, C24, FALSE)</f>
         <v>4.383675261853278E-2</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="9">
         <f t="shared" si="0"/>
         <v>6.1391666666666671</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="5">
         <v>9.0231944444444441</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="7" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="8">
         <v>7.4317129629629636E-2</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="7">
         <v>5</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="7">
         <f>_xlfn.NORM.DIST(D7, C23, C24, FALSE)</f>
         <v>4.9020846112334739E-2</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="9">
         <f t="shared" si="0"/>
         <v>1.7836111111111113</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="5">
         <v>7.2972685185185187</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="7" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="8">
         <v>0.24124999999999999</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="7">
         <v>6</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="7">
         <f>_xlfn.NORM.DIST(D8, C23, C24, FALSE)</f>
         <v>5.3558441055453709E-2</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="9">
         <f t="shared" si="0"/>
         <v>5.79</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="5">
         <v>8.9649999999999999</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="7" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="A9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="8">
         <v>0.97932870370370373</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="7">
         <v>7</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="7">
         <f>_xlfn.NORM.DIST(D9, C23, C24, FALSE)</f>
         <v>5.7171521159556989E-2</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="9">
         <f t="shared" si="0"/>
         <v>23.503888888888888</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="5">
         <v>6.917314814814814</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="R9" s="4" t="s">
+      <c r="R9" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="S9" s="4" t="s">
+      <c r="S9" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="T9" s="4" t="s">
+      <c r="T9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="U9" s="4" t="s">
+      <c r="U9" s="1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="A10" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="8">
         <v>0.1736111111111111</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="7">
         <v>8</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="7">
         <f>_xlfn.NORM.DIST(D10, C23, C24, FALSE)</f>
         <v>5.9626080733623271E-2</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="9">
         <f t="shared" si="0"/>
         <v>4.1666666666666661</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="5">
         <v>9.6944444444444446</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="R10" s="4" t="s">
+      <c r="R10" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="S10" s="4" t="s">
+      <c r="S10" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="T10" s="5" t="s">
+      <c r="T10" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="U10" s="4" t="s">
+      <c r="U10" s="1" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="8">
         <v>0.26725694444444442</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="7">
         <v>9</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="7">
         <f>_xlfn.NORM.DIST(D11, C23, C24, FALSE)</f>
         <v>6.0757161486998508E-2</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="9">
         <f t="shared" si="0"/>
         <v>6.4141666666666666</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="5">
         <v>10.069027777777778</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="R11" s="4" t="s">
+      <c r="R11" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="S11" s="4" t="s">
+      <c r="S11" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="T11" s="4" t="s">
+      <c r="T11" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="U11" s="4" t="s">
+      <c r="U11" s="1" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="A12" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="8">
         <v>0.30555555555555558</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="7">
         <v>10</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="7">
         <f>_xlfn.NORM.DIST(D12, C23, C24, FALSE)</f>
         <v>6.0487186450927155E-2</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="9">
         <f t="shared" si="0"/>
         <v>7.3333333333333339</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="5">
         <v>8.2222222222222214</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="R12" s="4" t="s">
+      <c r="R12" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="S12" s="6">
+      <c r="S12" s="3">
         <v>1</v>
       </c>
-      <c r="T12" s="7" t="s">
+      <c r="T12" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="U12" s="4" t="s">
+      <c r="U12" s="1" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="A13" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="8">
         <v>0.6166666666666667</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="7">
         <v>11</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="7">
         <f>_xlfn.NORM.DIST(D13, C23, C24, FALSE)</f>
         <v>5.8834760210180449E-2</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="9">
         <f t="shared" si="0"/>
         <v>14.8</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="5">
         <v>4.9666666666666668</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13" s="7" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="A14" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="8">
         <v>0.92246527777777776</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="7">
         <v>12</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="7">
         <f>_xlfn.NORM.DIST(D14, C23, C24, FALSE)</f>
         <v>5.5912548458414646E-2</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="9">
         <f t="shared" si="0"/>
         <v>22.139166666666668</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="5">
         <v>6.689861111111111</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" s="7" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="A15" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="8">
         <v>0.20640046296296297</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="7">
         <v>13</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="7">
         <f>_xlfn.NORM.DIST(D15, C23, C24, FALSE)</f>
         <v>5.1914572645209558E-2</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="9">
         <f t="shared" si="0"/>
         <v>4.953611111111111</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="5">
         <v>7.825601851851852</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" s="7" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="8">
         <v>0.20371527777777779</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="7">
         <v>14</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="7">
         <f>_xlfn.NORM.DIST(D16, C23, C24, FALSE)</f>
         <v>4.7094910396608521E-2</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="9">
         <f t="shared" si="0"/>
         <v>4.8891666666666671</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G16" s="5">
         <v>9.5648611111111101</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="7" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="A17" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" s="8">
         <v>0.15690972222222221</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="7">
         <v>15</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="7">
         <f>_xlfn.NORM.DIST(D17, C23, C24, FALSE)</f>
         <v>4.1741049317978722E-2</v>
       </c>
-      <c r="F17" s="3">
+      <c r="F17" s="9">
         <f t="shared" si="0"/>
         <v>3.7658333333333331</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17" s="5">
         <v>7.6276388888888889</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17" s="7" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="A18" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18" s="8">
         <v>0.2522800925925926</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="7">
         <v>16</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="7">
         <f>_xlfn.NORM.DIST(D18, C23, C24, FALSE)</f>
         <v>3.6145767099709965E-2</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18" s="9">
         <f t="shared" si="0"/>
         <v>6.0547222222222228</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="5">
         <v>8.5091203703703702</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H18" s="7" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="A19" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19" s="8">
         <v>0.3</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="7">
         <v>17</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="7">
         <f>_xlfn.NORM.DIST(D19, C23, C24, FALSE)</f>
         <v>3.0581319867986272E-2</v>
       </c>
-      <c r="F19" s="3">
+      <c r="F19" s="9">
         <f t="shared" si="0"/>
         <v>7.1999999999999993</v>
       </c>
-      <c r="G19" s="9">
+      <c r="G19" s="5">
         <v>9.4499999999999993</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19" s="7" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="A20" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="8">
         <v>0.22863425925925926</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="7">
         <v>18</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="7">
         <f>_xlfn.NORM.DIST(D20, C23, C24, FALSE)</f>
         <v>2.5278988981672211E-2</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F20" s="9">
         <f t="shared" si="0"/>
         <v>5.487222222222222</v>
       </c>
-      <c r="G20" s="9">
+      <c r="G20" s="5">
         <v>8.9145370370370376</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20" s="7" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="A21" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C21" s="8">
         <v>0.3082523148148148</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="7">
         <v>19</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="7">
         <f>_xlfn.NORM.DIST(D21, C23, C24, FALSE)</f>
         <v>2.0415869067398281E-2</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="9">
         <f t="shared" si="0"/>
         <v>7.3980555555555547</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21" s="5">
         <v>9.2330092592592585</v>
       </c>
-      <c r="H21" t="s">
+      <c r="H21" s="7" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D22">
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7">
         <v>20</v>
       </c>
-      <c r="E22">
+      <c r="E22" s="7">
         <f>_xlfn.NORM.DIST(D22, C23, C24, FALSE)</f>
         <v>1.6109450952465534E-2</v>
       </c>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
+      <c r="A23" s="7"/>
+      <c r="B23" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="3">
+      <c r="C23" s="12">
         <f>AVERAGE(F2:F21)</f>
         <v>9.3084166666666626</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="7">
         <v>21</v>
       </c>
-      <c r="E23">
+      <c r="E23" s="7">
         <f>_xlfn.NORM.DIST(D23, C23, C24, FALSE)</f>
         <v>1.2419333855944766E-2</v>
       </c>
-      <c r="G23" s="3">
+      <c r="F23" s="7"/>
+      <c r="G23" s="9">
         <f>AVERAGE(G2:G21)</f>
         <v>8.2264027777777766</v>
       </c>
+      <c r="H23" s="7"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
+      <c r="A24" s="7"/>
+      <c r="B24" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="3">
+      <c r="C24" s="13">
         <f>_xlfn.STDEV.P(F2:F21)</f>
         <v>6.5589218011554982</v>
       </c>
-      <c r="D24">
+      <c r="D24" s="7">
         <v>22</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="7">
         <f>_xlfn.NORM.DIST(D24, C23, C24, FALSE)</f>
         <v>9.3544996021318171E-3</v>
       </c>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D25">
+      <c r="A25" s="7"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7">
         <v>23</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="7">
         <f>_xlfn.NORM.DIST(D25, C23, C24, FALSE)</f>
         <v>6.8841054739413148E-3</v>
       </c>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D26">
+      <c r="A26" s="7"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7">
         <v>24</v>
       </c>
-      <c r="E26">
+      <c r="E26" s="7">
         <f>_xlfn.NORM.DIST(D26, C23, C24, FALSE)</f>
         <v>4.9497032959050285E-3</v>
       </c>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D27">
+      <c r="A27" s="7"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7">
         <v>25</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="7">
         <f>_xlfn.NORM.DIST(D27, C23, C24, FALSE)</f>
         <v>3.4770866463822328E-3</v>
       </c>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="11"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="10"/>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="10"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+    </row>
+    <row r="33" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E33" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>